<commit_message>
fix write back of conditional formating
</commit_message>
<xml_diff>
--- a/src/test/ErrorsAndWarnings.xlsx
+++ b/src/test/ErrorsAndWarnings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Git\node-projects\ExcelForge\src\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A8A0FD-D41F-474A-AFEF-43A3E8794407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FFD8915-D303-4C09-B3E0-20B85BF754C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="31036" windowHeight="18825" xr2:uid="{430383D8-2DF1-414F-83B0-55DD456A3C4D}"/>
+    <workbookView xWindow="4853" yWindow="3803" windowWidth="23129" windowHeight="13695" xr2:uid="{430383D8-2DF1-414F-83B0-55DD456A3C4D}"/>
   </bookViews>
   <sheets>
     <sheet name="ErrorsAndWarnings" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Comment</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>Time</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>Warning</t>
   </si>
 </sst>
 </file>
@@ -620,10 +626,16 @@
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" s="4"/>
       <c r="B2" s="5"/>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" s="4"/>
       <c r="B3" s="5"/>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" s="4"/>

</xml_diff>